<commit_message>
Deploy Atlas site from cecafa5bba42ed856a2a63ef8c2f7e9c124e2dc1
</commit_message>
<xml_diff>
--- a/downloads/formulas/adaptive-metrics-and-visual-management.xlsx
+++ b/downloads/formulas/adaptive-metrics-and-visual-management.xlsx
@@ -25,8 +25,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +44,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000000FF"/>
     </font>
   </fonts>
   <fills count="6">
@@ -84,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -97,6 +102,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1407,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1472,24 +1489,36 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Control chart</t>
+          <t>Lead-time boundaries</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Limits are supplied illustrative inputs. No control-limit formula is published.</t>
+          <t>Customer, commitment, procurement, schedule lead, cycle time, work item age, waiting, and WIP are kept distinct. Date examples use elapsed calendar days: end date minus start date.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>Control chart</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Limits are supplied illustrative inputs. No control-limit formula is published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>July 2026 PMI Lessons 5 and 7; Scrum Guide 2020; Kanban Guide May 2025.</t>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>July 2026 PMI Lessons 5 and 7; verified Atlas schedule and procurement sources; Scrum Guide 2020; Kanban Guide May 2025.</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1683,7 +1712,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Lead Time</t>
+          <t>Customer Lead Time</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1693,7 +1722,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Lead time = delivery time - defined request or commitment time</t>
+          <t>Customer lead time = delivery date - customer request date</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1703,61 +1732,61 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Name the start convention; Do not compare incompatible endpoints</t>
+          <t>Name both boundaries; Do not call WIP duration customer lead time unless work start is also the selected request boundary</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>SRC-PMI-COURSE-LESSON-7-2026</t>
+          <t>SRC-PMI-COURSE-LESSON-7-2026; SRC-CONFLUENCE-SCHEDULE</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>ADM-WIP-001</t>
+          <t>ADM-LEAD-002</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Work in Progress</t>
+          <t>Commitment Lead Time</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>flow metric</t>
+          <t>time measure</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>WIP = count of items started and not finished</t>
+          <t>Commitment lead time = delivery date - commitment date</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Work items.</t>
+          <t>Elapsed calendar or working time under a stated convention.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>A limit without an explicit workflow policy is insufficient</t>
+          <t>Name the commitment policy; Do not assume a tool column defines commitment universally</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>SRC-PMI-COURSE-LESSON-7-2026; SRC-KANBAN-GUIDE</t>
+          <t>SRC-PMI-COURSE-LESSON-7-2026; SRC-CONFLUENCE-SCHEDULE</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>ADM-AGE-001</t>
+          <t>ADM-PROC-LEAD-001</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Work Item Age</t>
+          <t>Procurement Lead Time</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1767,202 +1796,202 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Work item age = current time - workflow start time</t>
+          <t>Procurement lead time = available or delivery date - order or requisition date</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Elapsed time.</t>
+          <t>Elapsed calendar or working time under a stated convention.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Age is a signal for investigation; not blame</t>
+          <t>Do not confuse procurement elapsed time with a precedence relationship lead</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>SRC-KANBAN-GUIDE</t>
+          <t>SRC-CONFLUENCE-RISK; SRC-CONFLUENCE-SCHEDULE</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>ADM-BURN-001</t>
+          <t>ADM-SCH-LEAD-001</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Burn Charts</t>
+          <t>Schedule Lead</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>cumulative measure</t>
+          <t>time measure</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Remaining work = total scope - completed work</t>
+          <t>Schedule lead = permitted predecessor-successor overlap stated on the precedence relationship</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Consistent work units over time.</t>
+          <t>Working time in the schedule calendar.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Do not hide scope change; Incomplete work remains in the total</t>
+          <t>Not customer lead time; Not procurement lead time; Do not reproduce a full network calculation here</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>SRC-PMI-COURSE-LESSON-5-2026; SRC-PMI-COURSE-LESSON-7-2026</t>
+          <t>SRC-CONFLUENCE-SCHEDULE</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>ADM-CFD-001</t>
+          <t>ADM-WIP-001</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Cumulative Flow Diagram</t>
+          <t>Work in Progress</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>cumulative measure</t>
+          <t>flow metric</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Each boundary equals the cumulative count at or beyond a workflow state</t>
+          <t>WIP = count of items started and not finished</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Work items over time.</t>
+          <t>Work items.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>One diagram does not prove a cause</t>
+          <t>A limit without an explicit workflow policy is insufficient</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>SRC-PMI-COURSE-LESSON-5-2026; SRC-PMI-COURSE-LESSON-7-2026</t>
+          <t>SRC-PMI-COURSE-LESSON-7-2026; SRC-KANBAN-GUIDE</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ADM-BOARD-001</t>
+          <t>ADM-AGE-001</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Task Board or Kanban Board</t>
+          <t>Work Item Age</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>visual-management tool</t>
+          <t>time measure</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Work item age = current time - workflow start time</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Work items by state.</t>
+          <t>Elapsed time.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Not every task board is a complete Kanban system</t>
+          <t>Age is a signal for investigation; not blame</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>SRC-PMI-COURSE-LESSON-5-2026; SRC-PMI-COURSE-LESSON-7-2026; SRC-KANBAN-GUIDE</t>
+          <t>SRC-KANBAN-GUIDE</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ADM-CONTROL-001</t>
+          <t>ADM-BURN-001</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Control Chart</t>
+          <t>Burn Charts</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>process-stability measure</t>
+          <t>cumulative measure</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Mean = sum of observations / number of observations; control limits are supplied illustrative inputs, not calculated here.</t>
+          <t>Remaining work = total scope - completed work</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Same unit as the plotted process measure.</t>
+          <t>Consistent work units over time.</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Do not publish or infer an unsupported limit formula</t>
+          <t>Do not hide scope change; Incomplete work remains in the total</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>SRC-PMI-COURSE-LESSON-7-2026</t>
+          <t>SRC-PMI-COURSE-LESSON-5-2026; SRC-PMI-COURSE-LESSON-7-2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>ADM-RAD-001</t>
+          <t>ADM-CFD-001</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Information Radiator</t>
+          <t>Cumulative Flow Diagram</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>visual-management tool</t>
+          <t>cumulative measure</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Each boundary equals the cumulative count at or beyond a workflow state</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Not applicable.</t>
+          <t>Work items over time.</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Visibility does not make stale information useful</t>
+          <t>One diagram does not prove a cause</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1974,35 +2003,146 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>ADM-BOARD-001</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Task Board or Kanban Board</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>visual-management tool</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Work items by state.</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Not every task board is a complete Kanban system</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>SRC-PMI-COURSE-LESSON-5-2026; SRC-PMI-COURSE-LESSON-7-2026; SRC-KANBAN-GUIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ADM-CONTROL-001</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Control Chart</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>process-stability measure</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Mean = sum of observations / number of observations; control limits are supplied illustrative inputs, not calculated here.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Same unit as the plotted process measure.</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Do not publish or infer an unsupported limit formula</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>SRC-PMI-COURSE-LESSON-7-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ADM-RAD-001</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Information Radiator</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>visual-management tool</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Visibility does not make stale information useful</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>SRC-PMI-COURSE-LESSON-5-2026; SRC-PMI-COURSE-LESSON-7-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
           <t>ADM-IMP-001</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Impediment List and Visualization</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>impediment measure</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Age = current date - identified date</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Impediment count and elapsed age.</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Scrum Master accountability does not mean personal removal of every impediment; Do not penalize a team for reporting impediments</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>SRC-PMI-COURSE-LESSON-5-2026; SRC-PMI-COURSE-LESSON-7-2026</t>
         </is>
@@ -2936,16 +3076,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2958,72 +3099,413 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Example / result</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Request day</t>
+          <t>Boundary 1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Work starts</t>
+          <t>Boundary 2</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Delivery day</t>
+          <t>Duration</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Lead time</t>
+          <t>Meaning</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Cycle time</t>
+          <t>Waiting / effect</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Age / risk</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Convention / distinction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>PREDICTIVE PROCUREMENT LEAD TIME</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Order date</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Delivery date</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Lead time days</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Schedule use</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Distinction</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>specialized infrastructure appliance</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>46127</v>
+      </c>
+      <c r="D4" s="8">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Availability constraint before installation</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Not a precedence lead</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>PREDICTIVE SCHEDULE LEAD</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Predecessor</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Successor</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Effect</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Distinction</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Coding to Testing</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Coding</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>working days</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Testing may start before Coding finishes</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Coordination or rework</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Not customer lead time</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>ADAPTIVE MILESTONES</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Request</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Commitment</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Started</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Finished</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Measurement date</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>SB-118</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>46143</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>46150</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>46152</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>46159</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>46162</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>46162</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>ADAPTIVE CALCULATIONS</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Customer lead</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Commitment lead</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Cycle / completed WIP duration</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Waiting before start</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Waiting after commitment</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Work item age</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
           <t>Convention</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>SB-118</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="E3" s="3">
-        <f>D3-B3</f>
-        <v/>
-      </c>
-      <c r="F3" s="3">
-        <f>D3-C3</f>
-        <v/>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Working-day fractions; compatible finish point</t>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="B13" s="8">
+        <f>G10-B10</f>
+        <v/>
+      </c>
+      <c r="C13" s="8">
+        <f>G10-C10</f>
+        <v/>
+      </c>
+      <c r="D13" s="8">
+        <f>F10-D10</f>
+        <v/>
+      </c>
+      <c r="E13" s="8">
+        <f>D10-B10</f>
+        <v/>
+      </c>
+      <c r="F13" s="8">
+        <f>D10-C10</f>
+        <v/>
+      </c>
+      <c r="G13" s="8">
+        <f>H10-D10</f>
+        <v/>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Elapsed calendar days: end date minus start date</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Status rule</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Request to delivery</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Commitment to delivery</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Started to finished</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Outside WIP</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Outside WIP</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Only while unfinished: In Progress on May 15</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Finished items use cycle time, not age</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>